<commit_message>
Add charts to the workbook and an Investment Considerations section to the report
- Textile_Peer_Comparison.xlsx: adds four comparison charts on the Peer
  Comparison sheet (P/E, OPM vs NPM, ROE vs ROCE, revenue vs net profit),
  built from the same cell ranges as the table so they stay in sync with the
  data.
- Textile_Industry_Equity_Research_Report.docx/.pdf: adds an Investment
  Considerations section that synthesizes the peer comparison data
  (valuation spread, profitability/returns, growth, leverage) — computed
  from the underlying figures rather than hardcoded, and framed as
  descriptive positioning within the peer set, not a recommendation.
- Table of contents page numbers re-verified against the actual rendered
  PDF after the new section shifted pagination.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014c24deaoFxEeriwm2WaAVx
</commit_message>
<xml_diff>
--- a/projects/textile-equity-research/Textile_Peer_Comparison.xlsx
+++ b/projects/textile-equity-research/Textile_Peer_Comparison.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="183">
   <si>
     <t xml:space="preserve">Indian Textile Industry</t>
   </si>
@@ -104,7 +104,7 @@
     <t xml:space="preserve">Sheets in this workbook</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Peer Comparison – valuation, profitability, growth and leverage across all 8 companies</t>
+    <t xml:space="preserve">1. Peer Comparison – valuation, profitability, growth and leverage across all 8 companies, with comparison charts</t>
   </si>
   <si>
     <t xml:space="preserve">2. Industry Overview – market size, export data, demand drivers, risks and government policy</t>
@@ -267,6 +267,9 @@
   </si>
   <si>
     <t xml:space="preserve">Median</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peer Comparison Charts</t>
   </si>
   <si>
     <t xml:space="preserve">Indian Textile &amp; Apparel Industry – Overview</t>
@@ -786,15 +789,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\₹#,##0.00"/>
     <numFmt numFmtId="166" formatCode="\₹#,##0"/>
     <numFmt numFmtId="167" formatCode="0.0\x"/>
     <numFmt numFmtId="168" formatCode="0.0%"/>
     <numFmt numFmtId="169" formatCode="0.00\x"/>
+    <numFmt numFmtId="170" formatCode="0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -890,6 +894,26 @@
       <family val="2"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="9"/>
       <color rgb="FF0563C1"/>
       <name val="Arial"/>
@@ -921,13 +945,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFF9F9F9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E2F3"/>
-        <bgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -980,7 +1004,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1117,6 +1141,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1129,11 +1157,11 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1145,7 +1173,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1175,15 +1203,15 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>
-      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFC0504D"/>
+      <rgbColor rgb="FFF9F9F9"/>
       <rgbColor rgb="FFF2F2F2"/>
-      <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0563C1"/>
-      <rgbColor rgb="FFD9E2F3"/>
+      <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -1193,14 +1221,14 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFD9E2F3"/>
       <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF4F81BD"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
@@ -1219,6 +1247,1861 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Valuation – P/E by Company</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Peer Comparison'!G4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>P/E (x)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4f81bd"/>
+            </a:solidFill>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="f9f9f9"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="0.0\x" sourceLinked="1"/>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Peer Comparison'!$A$5:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Vardhman Textiles Ltd</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Trident Limited</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Welspun Living Ltd</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Raymond Lifestyle Ltd</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Arvind Limited</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>K.P.R. Mill Limited</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Page Industries Limited</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Gokaldas Exports Ltd</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Peer Comparison'!$G$5:$G$12</c:f>
+              <c:numCache>
+                <c:formatCode>0.0\x</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>21.02</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>33.55</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>53.14</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>102.1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>36.3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>41.6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>55.64</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>58.9</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="150"/>
+        <c:overlap val="0"/>
+        <c:axId val="32261311"/>
+        <c:axId val="72515392"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="32261311"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="72515392"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="72515392"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>P/E (x)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.0\x" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="32261311"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Profitability – OPM vs NPM</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Peer Comparison'!M4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>OPM (%)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4f81bd"/>
+            </a:solidFill>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="f9f9f9"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="0%" sourceLinked="1"/>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Peer Comparison'!$A$5:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Vardhman Textiles Ltd</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Trident Limited</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Welspun Living Ltd</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Raymond Lifestyle Ltd</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Arvind Limited</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>K.P.R. Mill Limited</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Page Industries Limited</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Gokaldas Exports Ltd</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Peer Comparison'!$M$5:$M$12</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.151</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.1404</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.0917</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.114</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.114</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.2065</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.22</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.096</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Peer Comparison'!N4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>NPM (%)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="c0504d"/>
+            </a:solidFill>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="f9f9f9"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="0%" sourceLinked="1"/>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Peer Comparison'!$A$5:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Vardhman Textiles Ltd</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Trident Limited</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Welspun Living Ltd</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Raymond Lifestyle Ltd</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Arvind Limited</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>K.P.R. Mill Limited</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Page Industries Limited</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Gokaldas Exports Ltd</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Peer Comparison'!$N$5:$N$12</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.075</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.0556</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.0227</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.0067</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.0459</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.1277</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.146</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.0251</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="150"/>
+        <c:overlap val="0"/>
+        <c:axId val="18804417"/>
+        <c:axId val="22567182"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="18804417"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="22567182"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="22567182"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Margin (%)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0%" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="18804417"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Returns – ROE vs ROCE</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Peer Comparison'!O4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>ROE (%)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4f81bd"/>
+            </a:solidFill>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="f9f9f9"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="0%" sourceLinked="1"/>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Peer Comparison'!$A$5:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Vardhman Textiles Ltd</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Trident Limited</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Welspun Living Ltd</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Raymond Lifestyle Ltd</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Arvind Limited</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>K.P.R. Mill Limited</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Page Industries Limited</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Gokaldas Exports Ltd</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Peer Comparison'!$O$5:$O$12</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.0829</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.0961</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.0451</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.0083</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.0934</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.157</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.476</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.071</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Peer Comparison'!P4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>ROCE (%)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="c0504d"/>
+            </a:solidFill>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="f9f9f9"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="0%" sourceLinked="1"/>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Peer Comparison'!$A$5:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Vardhman Textiles Ltd</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Trident Limited</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Welspun Living Ltd</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Raymond Lifestyle Ltd</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Arvind Limited</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>K.P.R. Mill Limited</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Page Industries Limited</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Gokaldas Exports Ltd</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Peer Comparison'!$P$5:$P$12</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>0.0886</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.1073</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.058</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.0133</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.1553</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.196</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.682</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.086</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="150"/>
+        <c:overlap val="0"/>
+        <c:axId val="44587787"/>
+        <c:axId val="91623867"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="44587787"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="91623867"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="91623867"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Return (%)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0%" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="44587787"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Growth – Revenue vs Net Profit (₹ Cr)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Peer Comparison'!K4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Revenue (₹ Cr)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4f81bd"/>
+            </a:solidFill>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="f9f9f9"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="\₹#,##0" sourceLinked="1"/>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Peer Comparison'!$A$5:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Vardhman Textiles Ltd</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Trident Limited</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Welspun Living Ltd</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Raymond Lifestyle Ltd</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Arvind Limited</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>K.P.R. Mill Limited</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Page Industries Limited</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Gokaldas Exports Ltd</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Peer Comparison'!$K$5:$K$12</c:f>
+              <c:numCache>
+                <c:formatCode>\₹#,##0</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>10092.53</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6775</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9399.11</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6888</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9303.19</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6784</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>5246.8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3987.64</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Peer Comparison'!L4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Net Profit (₹ Cr)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="c0504d"/>
+            </a:solidFill>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="f9f9f9"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="\₹#,##0" sourceLinked="1"/>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Peer Comparison'!$A$5:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Vardhman Textiles Ltd</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Trident Limited</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Welspun Living Ltd</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Raymond Lifestyle Ltd</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Arvind Limited</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>K.P.R. Mill Limited</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Page Industries Limited</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Gokaldas Exports Ltd</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Peer Comparison'!$L$5:$L$12</c:f>
+              <c:numCache>
+                <c:formatCode>\₹#,##0</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>753.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>377</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>212.89</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46.17</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>426.97</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>866.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>763.8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>100.13</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="150"/>
+        <c:overlap val="0"/>
+        <c:axId val="73663433"/>
+        <c:axId val="20693533"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="73663433"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="20693533"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="20693533"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Amount (₹ Cr)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="\₹#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="73663433"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>838440</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>96480</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>108000</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="0" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="3591000"/>
+        <a:ext cx="7919640" cy="3239640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>838440</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>540720</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>108000</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="14135040" y="3591000"/>
+        <a:ext cx="7919640" cy="3239640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>106560</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>96480</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>108000</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 3"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="7210440"/>
+        <a:ext cx="7919640" cy="3239640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>106560</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>540720</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>108000</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 4"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="14135040" y="7210440"/>
+        <a:ext cx="7919640" cy="3239640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1474,7 +3357,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -2287,6 +4170,11 @@
         <v>0.62025</v>
       </c>
     </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="34" t="s">
+        <v>62</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:U1"/>
@@ -2299,7 +4187,8 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -2317,420 +4206,420 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B1" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="34" t="s">
-        <v>63</v>
-      </c>
-      <c r="B3" s="35" t="s">
+      <c r="A3" s="35" t="s">
         <v>64</v>
       </c>
+      <c r="B3" s="36" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="34" t="s">
-        <v>65</v>
-      </c>
-      <c r="B4" s="35" t="s">
+      <c r="A4" s="35" t="s">
         <v>66</v>
       </c>
+      <c r="B4" s="36" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="120" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="34" t="s">
-        <v>67</v>
-      </c>
-      <c r="B5" s="35" t="s">
+      <c r="A5" s="35" t="s">
         <v>68</v>
       </c>
+      <c r="B5" s="36" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="225" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="34" t="s">
-        <v>69</v>
-      </c>
-      <c r="B6" s="35" t="s">
+      <c r="A6" s="35" t="s">
         <v>70</v>
       </c>
+      <c r="B6" s="36" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="34" t="s">
-        <v>71</v>
-      </c>
-      <c r="B7" s="35" t="s">
+      <c r="A7" s="35" t="s">
         <v>72</v>
       </c>
+      <c r="B7" s="36" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="255" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="B8" s="35" t="s">
+      <c r="A8" s="35" t="s">
         <v>74</v>
+      </c>
+      <c r="B8" s="36" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B10" s="27"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B11" s="35" t="s">
+      <c r="A11" s="37" t="s">
         <v>77</v>
       </c>
+      <c r="B11" s="36" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B12" s="35" t="s">
-        <v>78</v>
+      <c r="A12" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" s="36" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B13" s="35" t="s">
-        <v>79</v>
+      <c r="A13" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" s="36" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B14" s="35" t="s">
-        <v>80</v>
+      <c r="A14" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B14" s="36" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B15" s="35" t="s">
-        <v>81</v>
+      <c r="A15" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B15" s="36" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B16" s="35" t="s">
-        <v>82</v>
+      <c r="A16" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" s="36" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B17" s="35" t="s">
-        <v>83</v>
+      <c r="A17" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" s="36" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B18" s="35" t="s">
-        <v>84</v>
+      <c r="A18" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B18" s="36" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="27" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B20" s="27"/>
     </row>
     <row r="21" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B21" s="35" t="s">
-        <v>86</v>
+      <c r="A21" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="36" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B22" s="35" t="s">
-        <v>87</v>
+      <c r="A22" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B22" s="36" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B23" s="35" t="s">
-        <v>88</v>
+      <c r="A23" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B23" s="36" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B24" s="35" t="s">
-        <v>89</v>
+      <c r="A24" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" s="36" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B25" s="35" t="s">
-        <v>90</v>
+      <c r="A25" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" s="36" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B26" s="35" t="s">
-        <v>91</v>
+      <c r="A26" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B26" s="36" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B27" s="35" t="s">
-        <v>92</v>
+      <c r="A27" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B27" s="36" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B28" s="35" t="s">
-        <v>93</v>
+      <c r="A28" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B28" s="36" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="27" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B30" s="27"/>
     </row>
     <row r="31" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B31" s="35" t="s">
-        <v>95</v>
+      <c r="A31" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B31" s="36" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B32" s="35" t="s">
-        <v>96</v>
+      <c r="A32" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B32" s="36" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B33" s="35" t="s">
-        <v>97</v>
+      <c r="A33" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B33" s="36" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B34" s="35" t="s">
-        <v>98</v>
+      <c r="A34" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" s="36" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B35" s="35" t="s">
-        <v>99</v>
+      <c r="A35" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B35" s="36" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B36" s="35" t="s">
-        <v>100</v>
+      <c r="A36" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B36" s="36" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="B37" s="35" t="s">
-        <v>101</v>
+      <c r="A37" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B37" s="36" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="37" t="s">
-        <v>103</v>
-      </c>
-      <c r="B41" s="37"/>
+      <c r="A41" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="B41" s="38"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="37" t="s">
-        <v>104</v>
-      </c>
-      <c r="B42" s="37"/>
+      <c r="A42" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="B42" s="38"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="37" t="s">
-        <v>105</v>
-      </c>
-      <c r="B43" s="37"/>
+      <c r="A43" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="B43" s="38"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="37" t="s">
-        <v>106</v>
-      </c>
-      <c r="B44" s="37"/>
+      <c r="A44" s="38" t="s">
+        <v>107</v>
+      </c>
+      <c r="B44" s="38"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="37" t="s">
-        <v>107</v>
-      </c>
-      <c r="B45" s="37"/>
+      <c r="A45" s="38" t="s">
+        <v>108</v>
+      </c>
+      <c r="B45" s="38"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="37" t="s">
-        <v>108</v>
-      </c>
-      <c r="B46" s="37"/>
+      <c r="A46" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="B46" s="38"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="37" t="s">
-        <v>109</v>
-      </c>
-      <c r="B47" s="37"/>
+      <c r="A47" s="38" t="s">
+        <v>110</v>
+      </c>
+      <c r="B47" s="38"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="37" t="s">
-        <v>110</v>
-      </c>
-      <c r="B48" s="37"/>
+      <c r="A48" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="B48" s="38"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="37" t="s">
-        <v>111</v>
-      </c>
-      <c r="B49" s="37"/>
+      <c r="A49" s="38" t="s">
+        <v>112</v>
+      </c>
+      <c r="B49" s="38"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="37" t="s">
-        <v>112</v>
-      </c>
-      <c r="B50" s="37"/>
+      <c r="A50" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="B50" s="38"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="37" t="s">
-        <v>113</v>
-      </c>
-      <c r="B51" s="37"/>
+      <c r="A51" s="38" t="s">
+        <v>114</v>
+      </c>
+      <c r="B51" s="38"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="37" t="s">
-        <v>114</v>
-      </c>
-      <c r="B52" s="37"/>
+      <c r="A52" s="38" t="s">
+        <v>115</v>
+      </c>
+      <c r="B52" s="38"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="37" t="s">
-        <v>115</v>
-      </c>
-      <c r="B53" s="37"/>
+      <c r="A53" s="38" t="s">
+        <v>116</v>
+      </c>
+      <c r="B53" s="38"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="B54" s="37"/>
+      <c r="A54" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="B54" s="38"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="37" t="s">
-        <v>117</v>
-      </c>
-      <c r="B55" s="37"/>
+      <c r="A55" s="38" t="s">
+        <v>118</v>
+      </c>
+      <c r="B55" s="38"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="37" t="s">
-        <v>118</v>
-      </c>
-      <c r="B56" s="37"/>
+      <c r="A56" s="38" t="s">
+        <v>119</v>
+      </c>
+      <c r="B56" s="38"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="37" t="s">
-        <v>119</v>
-      </c>
-      <c r="B57" s="37"/>
+      <c r="A57" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="B57" s="38"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="37" t="s">
-        <v>120</v>
-      </c>
-      <c r="B58" s="37"/>
+      <c r="A58" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="B58" s="38"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="37" t="s">
-        <v>121</v>
-      </c>
-      <c r="B59" s="37"/>
+      <c r="A59" s="38" t="s">
+        <v>122</v>
+      </c>
+      <c r="B59" s="38"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="37" t="s">
-        <v>122</v>
-      </c>
-      <c r="B60" s="37"/>
+      <c r="A60" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="B60" s="38"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="37" t="s">
-        <v>123</v>
-      </c>
-      <c r="B61" s="37"/>
+      <c r="A61" s="38" t="s">
+        <v>124</v>
+      </c>
+      <c r="B61" s="38"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="37" t="s">
-        <v>124</v>
-      </c>
-      <c r="B62" s="37"/>
+      <c r="A62" s="38" t="s">
+        <v>125</v>
+      </c>
+      <c r="B62" s="38"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="37" t="s">
-        <v>125</v>
-      </c>
-      <c r="B63" s="37"/>
+      <c r="A63" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="B63" s="38"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="37" t="s">
-        <v>126</v>
-      </c>
-      <c r="B64" s="37"/>
+      <c r="A64" s="38" t="s">
+        <v>127</v>
+      </c>
+      <c r="B64" s="38"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="37" t="s">
-        <v>127</v>
-      </c>
-      <c r="B65" s="37"/>
+      <c r="A65" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="B65" s="38"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="37" t="s">
-        <v>128</v>
-      </c>
-      <c r="B66" s="37"/>
+      <c r="A66" s="38" t="s">
+        <v>129</v>
+      </c>
+      <c r="B66" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="30">
@@ -2789,440 +4678,440 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B1" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="38"/>
+      <c r="B3" s="39"/>
     </row>
     <row r="4" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="B4" s="39" t="s">
+      <c r="A4" s="35" t="s">
         <v>131</v>
       </c>
+      <c r="B4" s="40" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="216" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="34" t="s">
-        <v>132</v>
-      </c>
-      <c r="B5" s="39" t="s">
+      <c r="A5" s="35" t="s">
         <v>133</v>
       </c>
+      <c r="B5" s="40" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="B6" s="39" t="s">
-        <v>134</v>
+      <c r="A6" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="40" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="B7" s="39" t="s">
+      <c r="A7" s="35" t="s">
         <v>136</v>
       </c>
+      <c r="B7" s="40" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="270" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="B8" s="39" t="s">
+      <c r="A8" s="35" t="s">
         <v>138</v>
       </c>
+      <c r="B8" s="40" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="240" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="40" t="s">
-        <v>102</v>
-      </c>
-      <c r="B9" s="41" t="s">
-        <v>139</v>
+      <c r="A9" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" s="42" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="38" t="s">
+      <c r="A11" s="39" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="38"/>
+      <c r="B11" s="39"/>
     </row>
     <row r="12" customFormat="false" ht="108" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="B12" s="39" t="s">
-        <v>140</v>
+      <c r="A12" s="35" t="s">
+        <v>131</v>
+      </c>
+      <c r="B12" s="40" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="189" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34" t="s">
-        <v>132</v>
-      </c>
-      <c r="B13" s="39" t="s">
-        <v>141</v>
+      <c r="A13" s="35" t="s">
+        <v>133</v>
+      </c>
+      <c r="B13" s="40" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="B14" s="39" t="s">
-        <v>142</v>
+      <c r="A14" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B14" s="40" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="B15" s="39" t="s">
-        <v>143</v>
+      <c r="A15" s="35" t="s">
+        <v>136</v>
+      </c>
+      <c r="B15" s="40" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="324" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="B16" s="39" t="s">
-        <v>144</v>
+      <c r="A16" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="B16" s="40" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="192" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="40" t="s">
-        <v>102</v>
-      </c>
-      <c r="B17" s="41" t="s">
-        <v>145</v>
+      <c r="A17" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17" s="42" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="38" t="s">
+      <c r="A19" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="38"/>
+      <c r="B19" s="39"/>
     </row>
     <row r="20" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="B20" s="39" t="s">
-        <v>146</v>
+      <c r="A20" s="35" t="s">
+        <v>131</v>
+      </c>
+      <c r="B20" s="40" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="216" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="34" t="s">
-        <v>132</v>
-      </c>
-      <c r="B21" s="39" t="s">
-        <v>147</v>
+      <c r="A21" s="35" t="s">
+        <v>133</v>
+      </c>
+      <c r="B21" s="40" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="B22" s="39" t="s">
-        <v>148</v>
+      <c r="A22" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="40" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="B23" s="39" t="s">
-        <v>149</v>
+      <c r="A23" s="35" t="s">
+        <v>136</v>
+      </c>
+      <c r="B23" s="40" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="283.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="B24" s="39" t="s">
-        <v>150</v>
+      <c r="A24" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="B24" s="40" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="396" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="40" t="s">
-        <v>102</v>
-      </c>
-      <c r="B25" s="41" t="s">
-        <v>151</v>
+      <c r="A25" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="B25" s="42" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="38" t="s">
+      <c r="A27" s="39" t="s">
         <v>45</v>
       </c>
-      <c r="B27" s="38"/>
+      <c r="B27" s="39"/>
     </row>
     <row r="28" customFormat="false" ht="202.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="B28" s="39" t="s">
-        <v>152</v>
+      <c r="A28" s="35" t="s">
+        <v>131</v>
+      </c>
+      <c r="B28" s="40" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="229.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="34" t="s">
-        <v>132</v>
-      </c>
-      <c r="B29" s="39" t="s">
-        <v>153</v>
+      <c r="A29" s="35" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="40" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="162" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="B30" s="39" t="s">
-        <v>154</v>
+      <c r="A30" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B30" s="40" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="B31" s="39" t="s">
-        <v>155</v>
+      <c r="A31" s="35" t="s">
+        <v>136</v>
+      </c>
+      <c r="B31" s="40" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="283.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="B32" s="39" t="s">
-        <v>156</v>
+      <c r="A32" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="B32" s="40" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="204" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="40" t="s">
-        <v>102</v>
-      </c>
-      <c r="B33" s="41" t="s">
-        <v>157</v>
+      <c r="A33" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="B33" s="42" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="38" t="s">
+      <c r="A35" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="B35" s="38"/>
+      <c r="B35" s="39"/>
     </row>
     <row r="36" customFormat="false" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="B36" s="39" t="s">
-        <v>158</v>
+      <c r="A36" s="35" t="s">
+        <v>131</v>
+      </c>
+      <c r="B36" s="40" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="216" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="34" t="s">
-        <v>132</v>
-      </c>
-      <c r="B37" s="39" t="s">
-        <v>159</v>
+      <c r="A37" s="35" t="s">
+        <v>133</v>
+      </c>
+      <c r="B37" s="40" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="162" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="B38" s="39" t="s">
-        <v>160</v>
+      <c r="A38" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B38" s="40" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="B39" s="39" t="s">
-        <v>161</v>
+      <c r="A39" s="35" t="s">
+        <v>136</v>
+      </c>
+      <c r="B39" s="40" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="378" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="B40" s="39" t="s">
-        <v>162</v>
+      <c r="A40" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="B40" s="40" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="288" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="40" t="s">
-        <v>102</v>
-      </c>
-      <c r="B41" s="41" t="s">
-        <v>163</v>
+      <c r="A41" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="B41" s="42" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="38" t="s">
+      <c r="A43" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="B43" s="38"/>
+      <c r="B43" s="39"/>
     </row>
     <row r="44" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="B44" s="39" t="s">
-        <v>164</v>
+      <c r="A44" s="35" t="s">
+        <v>131</v>
+      </c>
+      <c r="B44" s="40" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="189" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="34" t="s">
-        <v>132</v>
-      </c>
-      <c r="B45" s="39" t="s">
-        <v>165</v>
+      <c r="A45" s="35" t="s">
+        <v>133</v>
+      </c>
+      <c r="B45" s="40" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="148.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="B46" s="39" t="s">
-        <v>166</v>
+      <c r="A46" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B46" s="40" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="B47" s="39" t="s">
-        <v>167</v>
+      <c r="A47" s="35" t="s">
+        <v>136</v>
+      </c>
+      <c r="B47" s="40" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="297" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="B48" s="39" t="s">
-        <v>168</v>
+      <c r="A48" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="B48" s="40" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="204" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="40" t="s">
-        <v>102</v>
-      </c>
-      <c r="B49" s="41" t="s">
-        <v>169</v>
+      <c r="A49" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="B49" s="42" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="38" t="s">
+      <c r="A51" s="39" t="s">
         <v>54</v>
       </c>
-      <c r="B51" s="38"/>
+      <c r="B51" s="39"/>
     </row>
     <row r="52" customFormat="false" ht="175.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="B52" s="39" t="s">
-        <v>170</v>
+      <c r="A52" s="35" t="s">
+        <v>131</v>
+      </c>
+      <c r="B52" s="40" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="189" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="34" t="s">
-        <v>132</v>
-      </c>
-      <c r="B53" s="39" t="s">
-        <v>171</v>
+      <c r="A53" s="35" t="s">
+        <v>133</v>
+      </c>
+      <c r="B53" s="40" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="B54" s="39" t="s">
-        <v>172</v>
+      <c r="A54" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B54" s="40" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="40.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="B55" s="39" t="s">
-        <v>173</v>
+      <c r="A55" s="35" t="s">
+        <v>136</v>
+      </c>
+      <c r="B55" s="40" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="297" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="B56" s="39" t="s">
-        <v>174</v>
+      <c r="A56" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="B56" s="40" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="204" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="40" t="s">
-        <v>102</v>
-      </c>
-      <c r="B57" s="41" t="s">
-        <v>175</v>
+      <c r="A57" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="B57" s="42" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="38" t="s">
+      <c r="A59" s="39" t="s">
         <v>57</v>
       </c>
-      <c r="B59" s="38"/>
+      <c r="B59" s="39"/>
     </row>
     <row r="60" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="34" t="s">
-        <v>130</v>
-      </c>
-      <c r="B60" s="39" t="s">
-        <v>176</v>
+      <c r="A60" s="35" t="s">
+        <v>131</v>
+      </c>
+      <c r="B60" s="40" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="175.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="34" t="s">
-        <v>132</v>
-      </c>
-      <c r="B61" s="39" t="s">
-        <v>177</v>
+      <c r="A61" s="35" t="s">
+        <v>133</v>
+      </c>
+      <c r="B61" s="40" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="B62" s="39" t="s">
-        <v>178</v>
+      <c r="A62" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="B62" s="40" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="34" t="s">
-        <v>135</v>
-      </c>
-      <c r="B63" s="39" t="s">
-        <v>179</v>
+      <c r="A63" s="35" t="s">
+        <v>136</v>
+      </c>
+      <c r="B63" s="40" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="283.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="34" t="s">
-        <v>137</v>
-      </c>
-      <c r="B64" s="39" t="s">
-        <v>180</v>
+      <c r="A64" s="35" t="s">
+        <v>138</v>
+      </c>
+      <c r="B64" s="40" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="204" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="40" t="s">
-        <v>102</v>
-      </c>
-      <c r="B65" s="41" t="s">
-        <v>181</v>
+      <c r="A65" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="B65" s="42" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>

</xml_diff>